<commit_message>
Tiny Sparks Day 2: Learn Numbers 1–10 with Animals (Short)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -1429,7 +1429,7 @@
       </c>
       <c r="Q3" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R3" s="48">
@@ -1445,7 +1445,11 @@
       <c r="V3" s="15" t="n"/>
       <c r="W3" s="15" t="n"/>
       <c r="X3" s="20" t="n"/>
-      <c r="Y3" s="15" t="n"/>
+      <c r="Y3" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-07 → kids-shorts/tiny-sparks/numbers/day-002-learn-numbers-1-10-with-animals/output/day-002-sfx-music.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="15" t="n">

</xml_diff>

<commit_message>
Tiny Sparks Day 3: 10 Animals in English & French (long 16:9)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -1527,7 +1527,7 @@
       </c>
       <c r="Q4" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R4" s="48">
@@ -1543,7 +1543,11 @@
       <c r="V4" s="15" t="n"/>
       <c r="W4" s="15" t="n"/>
       <c r="X4" s="20" t="n"/>
-      <c r="Y4" s="15" t="n"/>
+      <c r="Y4" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-08 → kids-shorts/tiny-sparks/words/day-003-20-animals-in-english-and-french/output/day-003-sfx-music.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="15" t="n">

</xml_diff>

<commit_message>
Tiny Sparks Day 4: Rory the Lion Who Was Afraid of the Dark (long 16:9, new pacing)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -1625,7 +1625,7 @@
       </c>
       <c r="Q5" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R5" s="48">
@@ -1641,7 +1641,11 @@
       <c r="V5" s="15" t="n"/>
       <c r="W5" s="15" t="n"/>
       <c r="X5" s="20" t="n"/>
-      <c r="Y5" s="15" t="n"/>
+      <c r="Y5" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-08 → kids-shorts/tiny-sparks/animals/day-004-rory-the-lion-who-was-afraid-of-the-dark/output/day-004-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="15" t="n">

</xml_diff>

<commit_message>
Day 5: Why Is the Sky Blue? (Science for Kids #1, 75 s Short)
Mila asks, Leo guesses, Prof. Hoot models sunlight -> air -> blue scatters;
one word (SCATTER) with a your-turn pause, 3-card recap, Mars blue-sunset wow.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -1723,7 +1723,7 @@
       </c>
       <c r="Q6" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R6" s="48">
@@ -1739,7 +1739,11 @@
       <c r="V6" s="15" t="n"/>
       <c r="W6" s="15" t="n"/>
       <c r="X6" s="20" t="n"/>
-      <c r="Y6" s="15" t="n"/>
+      <c r="Y6" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/science/day-005-why-is-the-sky-blue/output/day-005-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="n">

</xml_diff>

<commit_message>
Day 6: Find the Missing Number (Puzzles #1, 85 s Short)
Three chalkboard number puzzles with 5 s think timers, Leo's wrong tries,
counting-dot reveals and a 3-star YOU score strip.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -1821,7 +1821,7 @@
       </c>
       <c r="Q7" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R7" s="48">
@@ -1837,7 +1837,11 @@
       <c r="V7" s="15" t="n"/>
       <c r="W7" s="15" t="n"/>
       <c r="X7" s="20" t="n"/>
-      <c r="Y7" s="15" t="n"/>
+      <c r="Y7" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/puzzles/day-006-find-the-missing-number/output/day-006-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="15" t="n">

</xml_diff>

<commit_message>
Day 7: Count from 1 to 10 Song (Songs #1, 2:45 16:9, original song)
Rendered, muxed with song.mp3, marked done. video-of-the-day: two-pass
fallback when a long video is still over the 30 MB send limit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -1919,7 +1919,7 @@
       </c>
       <c r="Q8" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R8" s="48">
@@ -1935,7 +1935,11 @@
       <c r="V8" s="15" t="n"/>
       <c r="W8" s="15" t="n"/>
       <c r="X8" s="20" t="n"/>
-      <c r="Y8" s="15" t="n"/>
+      <c r="Y8" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/songs/day-007-count-from-1-to-10-song/output/day-007-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="n">

</xml_diff>

<commit_message>
Day 8: The Boy Who Always Told the Truth (Moral Stories #1, 2:57 16:9)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -2017,7 +2017,7 @@
       </c>
       <c r="Q9" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R9" s="48">
@@ -2033,7 +2033,11 @@
       <c r="V9" s="15" t="n"/>
       <c r="W9" s="15" t="n"/>
       <c r="X9" s="20" t="n"/>
-      <c r="Y9" s="15" t="n"/>
+      <c r="Y9" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/morals/day-008-the-boy-who-always-told-the-truth/output/day-008-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="n">

</xml_diff>

<commit_message>
Day 9: Counting 1–20 with Balloons (Numbers #2, 77 s Short)
Numbered balloons on each spoken number, a tied bunch of ten, 11-20 as 10 + k,
one balloon pops -> how many? -> 19.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -2115,7 +2115,7 @@
       </c>
       <c r="Q10" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R10" s="48">
@@ -2131,7 +2131,11 @@
       <c r="V10" s="15" t="n"/>
       <c r="W10" s="15" t="n"/>
       <c r="X10" s="20" t="n"/>
-      <c r="Y10" s="15" t="n"/>
+      <c r="Y10" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/numbers/day-009-counting-1-20-with-balloons/output/day-009-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="15" t="n">

</xml_diff>

<commit_message>
Day 10: 20 Colors in English and French (Words #2, 5:59 16:9)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -2213,7 +2213,7 @@
       </c>
       <c r="Q11" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R11" s="48">
@@ -2229,7 +2229,11 @@
       <c r="V11" s="15" t="n"/>
       <c r="W11" s="15" t="n"/>
       <c r="X11" s="20" t="n"/>
-      <c r="Y11" s="15" t="n"/>
+      <c r="Y11" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/words/day-010-20-colors-in-english-and-french/output/day-010-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="15" t="n">

</xml_diff>

<commit_message>
Day 11: Benny the Rabbit and the Lost Carrot (Animal Stories #2, 4:14 16:9)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -2311,7 +2311,7 @@
       </c>
       <c r="Q12" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R12" s="48">
@@ -2327,7 +2327,11 @@
       <c r="V12" s="15" t="n"/>
       <c r="W12" s="15" t="n"/>
       <c r="X12" s="20" t="n"/>
-      <c r="Y12" s="15" t="n"/>
+      <c r="Y12" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/animals/day-011-benny-the-rabbit-and-the-lost-carrot/output/day-011-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="15" t="n">

</xml_diff>

<commit_message>
Day 12: Why Does the Sun Shine? (Science #2, 80 s Short)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -2409,7 +2409,7 @@
       </c>
       <c r="Q13" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R13" s="48">
@@ -2425,7 +2425,11 @@
       <c r="V13" s="15" t="n"/>
       <c r="W13" s="15" t="n"/>
       <c r="X13" s="20" t="n"/>
-      <c r="Y13" s="15" t="n"/>
+      <c r="Y13" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/science/day-012-why-does-the-sun-shine/output/day-012-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="15" t="n">

</xml_diff>

<commit_message>
Day 13: Find the Missing Shape (Puzzles #2, 88 s Short)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -2507,7 +2507,7 @@
       </c>
       <c r="Q14" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R14" s="48">
@@ -2523,7 +2523,11 @@
       <c r="V14" s="15" t="n"/>
       <c r="W14" s="15" t="n"/>
       <c r="X14" s="20" t="n"/>
-      <c r="Y14" s="15" t="n"/>
+      <c r="Y14" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/puzzles/day-013-find-the-missing-shape/output/day-013-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="15" t="n">

</xml_diff>

<commit_message>
Day 14: Count from 1 to 20 Song (Songs #2, 2:16 16:9, original song)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -2605,7 +2605,7 @@
       </c>
       <c r="Q15" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R15" s="48">
@@ -2621,7 +2621,11 @@
       <c r="V15" s="15" t="n"/>
       <c r="W15" s="15" t="n"/>
       <c r="X15" s="20" t="n"/>
-      <c r="Y15" s="15" t="n"/>
+      <c r="Y15" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/songs/day-014-count-from-1-to-20-song/output/day-014-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="n">

</xml_diff>

<commit_message>
Day 15: Mila Learns to Say Please and Thank You (Stories #2, 2:51 16:9)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -2703,7 +2703,7 @@
       </c>
       <c r="Q16" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R16" s="48">
@@ -2719,7 +2719,11 @@
       <c r="V16" s="15" t="n"/>
       <c r="W16" s="15" t="n"/>
       <c r="X16" s="20" t="n"/>
-      <c r="Y16" s="15" t="n"/>
+      <c r="Y16" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/stories/day-015-mila-learns-to-say-please-and-thank-you/output/day-015-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="15" t="n">

</xml_diff>

<commit_message>
Day 16: Counting Apples 1–10 (Numbers #3, 63 s Short)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -2801,7 +2801,7 @@
       </c>
       <c r="Q17" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R17" s="48">
@@ -2817,7 +2817,11 @@
       <c r="V17" s="15" t="n"/>
       <c r="W17" s="15" t="n"/>
       <c r="X17" s="20" t="n"/>
-      <c r="Y17" s="15" t="n"/>
+      <c r="Y17" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/numbers/day-016-counting-apples-1-10/output/day-016-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="n">

</xml_diff>

<commit_message>
Day 17: Numbers 1–20 in English and French (Words #3, 5:51 16:9)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -2899,7 +2899,7 @@
       </c>
       <c r="Q18" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R18" s="48">
@@ -2915,7 +2915,11 @@
       <c r="V18" s="15" t="n"/>
       <c r="W18" s="15" t="n"/>
       <c r="X18" s="20" t="n"/>
-      <c r="Y18" s="15" t="n"/>
+      <c r="Y18" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/words/day-017-numbers-1-20-english-french/output/day-017-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="n">

</xml_diff>

<commit_message>
Day 18: Charlie the Monkey's Big Adventure (Animal Stories #3, 3:36 16:9)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -2997,7 +2997,7 @@
       </c>
       <c r="Q19" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R19" s="48">
@@ -3013,7 +3013,11 @@
       <c r="V19" s="15" t="n"/>
       <c r="W19" s="15" t="n"/>
       <c r="X19" s="20" t="n"/>
-      <c r="Y19" s="15" t="n"/>
+      <c r="Y19" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/animals/day-018-charlie-the-monkey-s-big-adventure/output/day-018-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="15" t="n">

</xml_diff>

<commit_message>
Day 19: Why Does the Moon Glow? (Science #3, 75 s Short)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -3095,7 +3095,7 @@
       </c>
       <c r="Q20" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R20" s="48">
@@ -3111,7 +3111,11 @@
       <c r="V20" s="15" t="n"/>
       <c r="W20" s="15" t="n"/>
       <c r="X20" s="20" t="n"/>
-      <c r="Y20" s="15" t="n"/>
+      <c r="Y20" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/science/day-019-why-does-the-moon-glow/output/day-019-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="15" t="n">

</xml_diff>

<commit_message>
Day 20: Find the Missing Color (Puzzles #3, 90 s Short)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -3193,7 +3193,7 @@
       </c>
       <c r="Q21" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R21" s="48">
@@ -3209,7 +3209,11 @@
       <c r="V21" s="15" t="n"/>
       <c r="W21" s="15" t="n"/>
       <c r="X21" s="20" t="n"/>
-      <c r="Y21" s="15" t="n"/>
+      <c r="Y21" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/puzzles/day-020-find-the-missing-color/output/day-020-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="15" t="n">

</xml_diff>

<commit_message>
Day 21: Alphabet A–Z Song (Songs #3, 3:04 16:9, original song)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -3291,7 +3291,7 @@
       </c>
       <c r="Q22" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R22" s="48">
@@ -3307,7 +3307,11 @@
       <c r="V22" s="15" t="n"/>
       <c r="W22" s="15" t="n"/>
       <c r="X22" s="20" t="n"/>
-      <c r="Y22" s="15" t="n"/>
+      <c r="Y22" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/songs/day-021-alphabet-a-z-song/output/day-021-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="15" t="n">

</xml_diff>

<commit_message>
Day 22: The Girl Who Learned to Share (Moral Stories #2, 2:37 16:9)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -3389,7 +3389,7 @@
       </c>
       <c r="Q23" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R23" s="48">
@@ -3405,7 +3405,11 @@
       <c r="V23" s="15" t="n"/>
       <c r="W23" s="15" t="n"/>
       <c r="X23" s="20" t="n"/>
-      <c r="Y23" s="15" t="n"/>
+      <c r="Y23" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/morals/day-022-the-girl-who-learned-to-share/output/day-022-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="15" t="n">

</xml_diff>

<commit_message>
Day 23: Count the Cute Puppies (Numbers #4, 67 s Short) + new 'dog' Critter species
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -3487,7 +3487,7 @@
       </c>
       <c r="Q24" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R24" s="48">
@@ -3503,7 +3503,11 @@
       <c r="V24" s="15" t="n"/>
       <c r="W24" s="15" t="n"/>
       <c r="X24" s="20" t="n"/>
-      <c r="Y24" s="15" t="n"/>
+      <c r="Y24" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/numbers/day-023-count-the-cute-puppies/output/day-023-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="15" t="n">

</xml_diff>

<commit_message>
Day 24: Family Members in English and French (Words #4, 1:53 Short) — first episode in hero outfits
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -3585,7 +3585,7 @@
       </c>
       <c r="Q25" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R25" s="48">
@@ -3601,7 +3601,11 @@
       <c r="V25" s="15" t="n"/>
       <c r="W25" s="15" t="n"/>
       <c r="X25" s="20" t="n"/>
-      <c r="Y25" s="15" t="n"/>
+      <c r="Y25" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/words/day-024-family-members-english-french/output/day-024-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="15" t="n">

</xml_diff>

<commit_message>
Day 25 done: Emma the Elephant (5:09, new livelier kit) — calendar updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -3683,7 +3683,7 @@
       </c>
       <c r="Q26" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R26" s="48">
@@ -3699,7 +3699,11 @@
       <c r="V26" s="15" t="n"/>
       <c r="W26" s="15" t="n"/>
       <c r="X26" s="20" t="n"/>
-      <c r="Y26" s="15" t="n"/>
+      <c r="Y26" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/animals/day-025-emma-the-elephant-helps-her-friend/output/day-025-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="15" t="n">

</xml_diff>

<commit_message>
Day 26: Why Do We Have Day and Night? (Science #4, 1:52 Short, hero outfits)
Day→night meadow hook, spinning top-down Earth with day/night halves, our house riding the spin with a
sky window (good morning / good night), spin-like-Earth your-turn, flashlight + ball + sticker demo,
two-houses other-side-of-the-world, 3-card recap, one spin = one day, sunrise loop.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -3781,7 +3781,7 @@
       </c>
       <c r="Q27" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R27" s="48">
@@ -3797,7 +3797,11 @@
       <c r="V27" s="15" t="n"/>
       <c r="W27" s="15" t="n"/>
       <c r="X27" s="20" t="n"/>
-      <c r="Y27" s="15" t="n"/>
+      <c r="Y27" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-09 → kids-shorts/tiny-sparks/science/day-026-why-do-we-have-day-and-night/output/day-026-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="15" t="n">

</xml_diff>

<commit_message>
Day 27: Which Animal Doesn't Belong? (Puzzles #4, 1:38 Short, hero outfits)
Odd-one-out by sound (cats vs dog), by body (fur vs feathers: the owl), and a super puzzle under the
sea (fish vs lion); THINK timers, Leo's guesses, group tags on the answer, YOU score strip.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -3879,7 +3879,7 @@
       </c>
       <c r="Q28" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R28" s="48">
@@ -3895,7 +3895,11 @@
       <c r="V28" s="15" t="n"/>
       <c r="W28" s="15" t="n"/>
       <c r="X28" s="20" t="n"/>
-      <c r="Y28" s="15" t="n"/>
+      <c r="Y28" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-10 → kids-shorts/tiny-sparks/puzzles/day-027-which-animal-doesn-t-belong/output/day-027-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="15" t="n">

</xml_diff>

<commit_message>
Day 28: The Colors Song (Songs #4, 5:08 long 16:9, original song, hero outfits)
Original 94 bpm song (gen_song chant): chorus, 10 colour verses with your-turn echoes, a colour-mixing
bridge, a sung colour quiz (grey picture coloured in on the answer), a karaoke 'now you sing' chorus.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -3977,7 +3977,7 @@
       </c>
       <c r="Q29" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R29" s="48">
@@ -3993,7 +3993,11 @@
       <c r="V29" s="15" t="n"/>
       <c r="W29" s="15" t="n"/>
       <c r="X29" s="20" t="n"/>
-      <c r="Y29" s="15" t="n"/>
+      <c r="Y29" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-10 → kids-shorts/tiny-sparks/songs/day-028-colors-song/output/day-028-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="15" t="n">

</xml_diff>

<commit_message>
Day 29: Bobo Learns to Clean His Room (Stories #3, 5:03 long 16:9, hero outfits)
Messy room + lost ball, I-spy, the under-the-bed try (BOING), 3 tidy-up steps with items flying home on each
number, the ball found under the hat, messy again, 10-to-1 tidy-up race, chant x3, 7-question remember quiz.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -4075,7 +4075,7 @@
       </c>
       <c r="Q30" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R30" s="48">
@@ -4091,7 +4091,11 @@
       <c r="V30" s="15" t="n"/>
       <c r="W30" s="15" t="n"/>
       <c r="X30" s="20" t="n"/>
-      <c r="Y30" s="15" t="n"/>
+      <c r="Y30" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-10 → kids-shorts/tiny-sparks/stories/day-029-bobo-learns-to-clean-his-room/output/day-029-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="15" t="n">

</xml_diff>

<commit_message>
Day 30: Count the Colorful Fish (Numbers #5, 1:26 Short) + the new FISH rig
lib/kids/sea.tsx: <Fish> (shared face, wagging tail, fins, stripes/spots/rainbow patterns) + <Bubbles>;
Underwater life={false}; fish registered as a built rig. Episode: 10 fish counted 1-10 on fingers,
find the blue fish, count the striped fish (3), fast recount, swim-away loop. Hero outfits + bubble helmets.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -4173,7 +4173,7 @@
       </c>
       <c r="Q31" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R31" s="48">
@@ -4189,7 +4189,11 @@
       <c r="V31" s="15" t="n"/>
       <c r="W31" s="15" t="n"/>
       <c r="X31" s="20" t="n"/>
-      <c r="Y31" s="15" t="n"/>
+      <c r="Y31" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-10 → kids-shorts/tiny-sparks/numbers/day-030-count-the-colorful-fish/output/day-030-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="15" t="n">

</xml_diff>

<commit_message>
Day 31: Fruits in English and French (Words #5, 2:12 Short, hero outfits)
Six fruit word cards (EN -> your turn -> FR -> sentence), a strawberry quiz with a think timer,
and a 3x2 recap grid lit word by word in English then French.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -4271,7 +4271,7 @@
       </c>
       <c r="Q32" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R32" s="48">
@@ -4287,7 +4287,11 @@
       <c r="V32" s="15" t="n"/>
       <c r="W32" s="15" t="n"/>
       <c r="X32" s="20" t="n"/>
-      <c r="Y32" s="15" t="n"/>
+      <c r="Y32" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-10 → kids-shorts/tiny-sparks/words/day-031-fruits-english-french/output/day-031-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="15" t="n">

</xml_diff>

<commit_message>
Day 32: Sammy the Turtle Learns Patience (Animals #5, 5:07 long 16:9) + turtle species
critter.tsx: 'turtle' (shell dome with scutes, plastron, beak-like nose, little tail) and a 'tuck' prop
that hides the head + paws in the shell. Episode: guess-who shell, hide-in-your-shell turn, 3 true facts,
strawberry seed dug up too soon, 3 waiting tricks (breathing guide, play, 'I can wait!'), days passing,
sprout -> flower -> red berry, remember round, 'Good things take time' chant.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -4369,7 +4369,7 @@
       </c>
       <c r="Q33" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R33" s="48">
@@ -4385,7 +4385,11 @@
       <c r="V33" s="15" t="n"/>
       <c r="W33" s="15" t="n"/>
       <c r="X33" s="20" t="n"/>
-      <c r="Y33" s="15" t="n"/>
+      <c r="Y33" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-10 → kids-shorts/tiny-sparks/animals/day-032-sammy-the-turtle-learns-patience/output/day-032-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="15" t="n">

</xml_diff>

<commit_message>
Day 33: Why Do Seasons Change? (Science #5, 1:51 Short, hero outfits)
Season-tile hook, Leo's close/far misconception, a perspective orbit with a tilted Earth (summer when our
side leans in, winter when it leans away, fall/spring between), lean-like-the-Earth turn, the flashlight
straight vs tilted demo, opposite hemispheres, recap, and the birthday-lap wow fact.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -4467,7 +4467,7 @@
       </c>
       <c r="Q34" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R34" s="48">
@@ -4483,7 +4483,11 @@
       <c r="V34" s="15" t="n"/>
       <c r="W34" s="15" t="n"/>
       <c r="X34" s="20" t="n"/>
-      <c r="Y34" s="15" t="n"/>
+      <c r="Y34" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-10 → kids-shorts/tiny-sparks/science/day-033-why-do-seasons-change/output/day-033-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="15" t="n">

</xml_diff>

<commit_message>
Day 34: Which Object Doesn't Belong? (Puzzles #5, 1:41 Short, 3D look) — rendered, calendar 34/800
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -4565,7 +4565,7 @@
       </c>
       <c r="Q35" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R35" s="48">
@@ -4581,7 +4581,11 @@
       <c r="V35" s="15" t="n"/>
       <c r="W35" s="15" t="n"/>
       <c r="X35" s="20" t="n"/>
-      <c r="Y35" s="15" t="n"/>
+      <c r="Y35" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-21 → kids-shorts/tiny-sparks/puzzles/day-034-which-object-doesn-t-belong/output/day-034-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" s="15" t="n">

</xml_diff>

<commit_message>
Day 35: The Shapes Song (Songs #5, 5:02 long 16:9, original song, 3D look)
Original 96 bpm song (gen_song chant): chorus, 10 shape verses with your-turn echoes, a build-with-shapes
bridge (house, ice cream, snowman), a sung shape quiz with outline tracing, a karaoke chorus. Shapes are
3D-shaded (<Vol>) with faces.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -4663,7 +4663,7 @@
       </c>
       <c r="Q36" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R36" s="48">
@@ -4679,7 +4679,11 @@
       <c r="V36" s="15" t="n"/>
       <c r="W36" s="15" t="n"/>
       <c r="X36" s="20" t="n"/>
-      <c r="Y36" s="15" t="n"/>
+      <c r="Y36" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-21 → kids-shorts/tiny-sparks/songs/day-035-shapes-song/output/day-035-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="15" t="n">

</xml_diff>

<commit_message>
Day 36: The Greedy Little Monkey (Morals #3, 5:07 long 16:9, 3D look)
Aesop's hand-in-the-jar fable retold: Momo wants all the nuts, his fist gets stuck, the word GREEDY,
'take just a few', sorry + sharing on three leaf plates (count along), picnic, 'Take a little, share
a lot!', remember round, a share-the-bananas turn, chant.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -4761,7 +4761,7 @@
       </c>
       <c r="Q37" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R37" s="48">
@@ -4777,7 +4777,11 @@
       <c r="V37" s="15" t="n"/>
       <c r="W37" s="15" t="n"/>
       <c r="X37" s="20" t="n"/>
-      <c r="Y37" s="15" t="n"/>
+      <c r="Y37" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-21 → kids-shorts/tiny-sparks/morals/day-036-the-greedy-little-monkey/output/day-036-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="15" t="n">

</xml_diff>

<commit_message>
Day 38: Vegetables in English & French (Words #6, 2:16 Short 9:16, energy layer)
Garden hook (pull, pull, POP! a giant carrot), 6 word loops EN then FR with card bursts and snap zooms,
gags, a broccoli quiz, recap grid, theme bed + 33 SFX cues. WordCard shrinks long French words to fit.
Calendar: 38/800.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -4957,7 +4957,7 @@
       </c>
       <c r="Q39" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R39" s="48">
@@ -4973,7 +4973,11 @@
       <c r="V39" s="15" t="n"/>
       <c r="W39" s="15" t="n"/>
       <c r="X39" s="20" t="n"/>
-      <c r="Y39" s="15" t="n"/>
+      <c r="Y39" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-22 → kids-shorts/tiny-sparks/words/day-038-vegetables-english-french/output/day-038-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="15" t="n">

</xml_diff>

<commit_message>
Day 39: Oliver the Owl's First Flight (Animal Stories #6, 5:01 long 16:9, energy layer)
Guess-who tree hole, owl sound + 3 true facts (nocturnal, ~270° head turn, silent feathers), the
friendship story (flap, hop into the leaf pile, 1-2-3 fly; Oliver rescues Bella's balloon), night,
5-question remember round, chant. 67 SFX cues + theme bed. Thumbnail + 36 s Short. Calendar: 39/800.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -5055,7 +5055,7 @@
       </c>
       <c r="Q40" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R40" s="48">
@@ -5071,7 +5071,11 @@
       <c r="V40" s="15" t="n"/>
       <c r="W40" s="15" t="n"/>
       <c r="X40" s="20" t="n"/>
-      <c r="Y40" s="15" t="n"/>
+      <c r="Y40" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-22 → kids-shorts/tiny-sparks/animals/day-039-oliver-the-owl-s-first-flight/output/day-039-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="15" t="n">

</xml_diff>

<commit_message>
Day 40: What Are Clouds? (Science #6, 1:43 Short 9:16, energy layer)
Leo's cotton-candy guess, the water cycle by the sea (evaporation, tiny drops gather into a cloud, rain),
a breathe-on-a-cold-mirror demo with a grown-up, recap, wow fact (~80 elephants, USGS). Calendar: 40/800.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -5153,7 +5153,7 @@
       </c>
       <c r="Q41" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R41" s="48">
@@ -5169,7 +5169,11 @@
       <c r="V41" s="15" t="n"/>
       <c r="W41" s="15" t="n"/>
       <c r="X41" s="20" t="n"/>
-      <c r="Y41" s="15" t="n"/>
+      <c r="Y41" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-22 → kids-shorts/tiny-sparks/science/day-040-what-are-clouds/output/day-040-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="15" t="n">

</xml_diff>

<commit_message>
Day 41: Find the Different Animal (Puzzles #6, 1:32 Short 9:16, energy layer)
Observation puzzles: four kittens (one orange), four bunnies (one crown), super puzzle 'which bear is
Bobo?' (the red scarf). Think timers on the beat, Leo's guesses, snap-zoom reveals, score strip.
Calendar: 41/800.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -5251,7 +5251,7 @@
       </c>
       <c r="Q42" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R42" s="48">
@@ -5267,7 +5267,11 @@
       <c r="V42" s="15" t="n"/>
       <c r="W42" s="15" t="n"/>
       <c r="X42" s="20" t="n"/>
-      <c r="Y42" s="15" t="n"/>
+      <c r="Y42" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-22 → kids-shorts/tiny-sparks/puzzles/day-041-find-the-different-animal/output/day-041-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="15" t="n">

</xml_diff>

<commit_message>
Day 42: Days of the Week Song (Songs #6, 5:08 long 16:9, original song, energy layer)
The Week Train (engine + 7 rainbow cars lit as each day is sung), 7 day verses with your-turn echoes,
a 5-question train quiz (what comes after / before), the weekend bridge, a karaoke chorus and a slow
pass. Channel ident on the jingle + 16 SFX cues. Thumbnail + 48 s Short. Calendar: 42/800.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -5349,7 +5349,7 @@
       </c>
       <c r="Q43" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R43" s="48">
@@ -5365,7 +5365,11 @@
       <c r="V43" s="15" t="n"/>
       <c r="W43" s="15" t="n"/>
       <c r="X43" s="20" t="n"/>
-      <c r="Y43" s="15" t="n"/>
+      <c r="Y43" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-22 → kids-shorts/tiny-sparks/songs/day-042-days-of-the-week-song/output/day-042-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="15" t="n">

</xml_diff>

<commit_message>
Day 43: final mix, thumbnail, Short; mark rendered in the calendar
Rebalanced the SFX plan from the audit_sfx pass: accents that sit under
speech get +6 dB (they were masked), gap cues are capped so cheers,
dings and ticks stay within ~2 dB of the voice. Final: 5:06.8, 1080p,
620 kb/s two-pass, -16.1 LUFS. Thumbnail: the drippy rainbow, WAIT,
MILA!. Short: Count to Ten with Mila (38.9 s).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -5447,7 +5447,7 @@
       </c>
       <c r="Q44" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R44" s="48">
@@ -5463,7 +5463,11 @@
       <c r="V44" s="15" t="n"/>
       <c r="W44" s="15" t="n"/>
       <c r="X44" s="20" t="n"/>
-      <c r="Y44" s="15" t="n"/>
+      <c r="Y44" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-22 → kids-shorts/tiny-sparks/stories/day-043-the-day-mila-learned-patience/output/day-043-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="15" t="n">

</xml_diff>

<commit_message>
Day 44: Count the Farm Animals (Short) + the farm kit
Numbers & Math #7, 9:16, 1:29. Bobo knocks on the red barn, five farm
animals walk out one by one (moo, oink, baa, quack, cheep) and are
counted with rainbow badges, the big numeral and Mila's fingers; a
5 s think, a recount, then the duck leaves for a swim (5 - 1 = 4) and
comes back (4 + 1 = 5); the animals walk back in and the doors close
for a soft loop.

New kit: cow, sheep, chick and duck species in the Critter rig and
lib/kids/farm.tsx (Barn with opening doors, Fence, HayBale, a FarmYard
hill for 9:16, the farm animal specs) with the KidsFarmSheet model
sheet. Badge pops lead each spoken number by 0.1 s so the pop SFX sits
in the breath before the word instead of under it.

Also aligns every episode's upload-kit playlist names with
channel/PLAYLISTS.md (several notes used older names).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -5545,7 +5545,7 @@
       </c>
       <c r="Q45" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R45" s="48">
@@ -5561,7 +5561,11 @@
       <c r="V45" s="15" t="n"/>
       <c r="W45" s="15" t="n"/>
       <c r="X45" s="20" t="n"/>
-      <c r="Y45" s="15" t="n"/>
+      <c r="Y45" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-22 → kids-shorts/tiny-sparks/numbers/day-044-count-the-farm-animals/output/day-044-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="15" t="n">

</xml_diff>

<commit_message>
Day 45: School Objects in English and French (Short)
English/French Words #7, 9:16, 2:19. Bobo's overfull backpack goes
zip, zip, POP; six school things come back down onto their cards one
by one (pencil/le crayon, book/le livre, ruler/la règle, eraser/la
gomme, glue/la colle, backpack/le sac à dos), each said twice in each
language with a your-turn pause and a small gag; a quiz (which one is
the ruler?), a recap grid in English then French, and goodbye.

gen_voice: when a line's phonetic tts variant has as many words as its
caption text, the timed words now take the caption spelling. Before,
'le sac à dô' (needed because espeak reads 'dos' as English DOS)
leaked into the on-screen captions. The kids-words skill notes how to
check French phonemes for an (en) switch.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -5643,7 +5643,7 @@
       </c>
       <c r="Q46" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R46" s="48">
@@ -5659,7 +5659,11 @@
       <c r="V46" s="15" t="n"/>
       <c r="W46" s="15" t="n"/>
       <c r="X46" s="20" t="n"/>
-      <c r="Y46" s="15" t="n"/>
+      <c r="Y46" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-22 → kids-shorts/tiny-sparks/words/day-045-school-objects-english-french/output/day-045-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="15" t="n">

</xml_diff>

<commit_message>
Marathon #2: Days 46-49 in one 21-min kids video + calendar ticked
- compilations/marathon-02: plan/cmd/chapters, upload kit, thumbnail (output mp4 gitignored)
- Day 49 snowflake colour fix; Days 46-49 marked Rendered (49/800)

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -5741,7 +5741,7 @@
       </c>
       <c r="Q47" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R47" s="48">
@@ -5757,7 +5757,11 @@
       <c r="V47" s="15" t="n"/>
       <c r="W47" s="15" t="n"/>
       <c r="X47" s="20" t="n"/>
-      <c r="Y47" s="15" t="n"/>
+      <c r="Y47" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-30 → kids-shorts/tiny-sparks/animals/day-046-coco-the-penguin-finds-a-friend/output/day-046-sfx-tiny-sparks-bounce.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="15" t="n">
@@ -5835,7 +5839,7 @@
       </c>
       <c r="Q48" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R48" s="48">
@@ -5851,7 +5855,11 @@
       <c r="V48" s="15" t="n"/>
       <c r="W48" s="15" t="n"/>
       <c r="X48" s="20" t="n"/>
-      <c r="Y48" s="15" t="n"/>
+      <c r="Y48" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-30 → kids-shorts/tiny-sparks/science/day-047-how-does-rain-form/output/day-047-sfx-tiny-sparks-bounce.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="15" t="n">
@@ -5929,7 +5937,7 @@
       </c>
       <c r="Q49" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R49" s="48">
@@ -5945,7 +5953,11 @@
       <c r="V49" s="15" t="n"/>
       <c r="W49" s="15" t="n"/>
       <c r="X49" s="20" t="n"/>
-      <c r="Y49" s="15" t="n"/>
+      <c r="Y49" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-30 → kids-shorts/tiny-sparks/puzzles/day-048-find-the-different-shape/output/day-048-sfx-tiny-sparks-bounce.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="15" t="n">
@@ -6023,7 +6035,7 @@
       </c>
       <c r="Q50" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R50" s="48">
@@ -6039,7 +6051,11 @@
       <c r="V50" s="15" t="n"/>
       <c r="W50" s="15" t="n"/>
       <c r="X50" s="20" t="n"/>
-      <c r="Y50" s="15" t="n"/>
+      <c r="Y50" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-30 → kids-shorts/tiny-sparks/songs/day-049-months-of-the-year-song/output/day-049-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="15" t="n">

</xml_diff>

<commit_message>
Marathon #3: Days 50-53 in one 20-min video + calendar ticked (53/800)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -6133,7 +6133,7 @@
       </c>
       <c r="Q51" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R51" s="48">
@@ -6149,7 +6149,11 @@
       <c r="V51" s="15" t="n"/>
       <c r="W51" s="15" t="n"/>
       <c r="X51" s="20" t="n"/>
-      <c r="Y51" s="15" t="n"/>
+      <c r="Y51" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-30 → kids-shorts/tiny-sparks/morals/day-050-the-kind-little-rabbit/output/day-050-sfx-tiny-sparks-bounce.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="15" t="n">
@@ -6227,7 +6231,7 @@
       </c>
       <c r="Q52" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R52" s="48">
@@ -6243,7 +6247,11 @@
       <c r="V52" s="15" t="n"/>
       <c r="W52" s="15" t="n"/>
       <c r="X52" s="20" t="n"/>
-      <c r="Y52" s="15" t="n"/>
+      <c r="Y52" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-30 → kids-shorts/tiny-sparks/numbers/day-051-count-the-butterflies/output/day-051-sfx-tiny-sparks-bounce.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="15" t="n">
@@ -6321,7 +6329,7 @@
       </c>
       <c r="Q53" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R53" s="48">
@@ -6337,7 +6345,11 @@
       <c r="V53" s="15" t="n"/>
       <c r="W53" s="15" t="n"/>
       <c r="X53" s="20" t="n"/>
-      <c r="Y53" s="15" t="n"/>
+      <c r="Y53" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-30 → kids-shorts/tiny-sparks/words/day-052-toys-english-french/output/day-052-sfx-tiny-sparks-bounce.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="15" t="n">
@@ -6415,7 +6427,7 @@
       </c>
       <c r="Q54" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R54" s="48">
@@ -6431,7 +6443,11 @@
       <c r="V54" s="15" t="n"/>
       <c r="W54" s="15" t="n"/>
       <c r="X54" s="20" t="n"/>
-      <c r="Y54" s="15" t="n"/>
+      <c r="Y54" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-30 → kids-shorts/tiny-sparks/animals/day-053-max-the-dog-saves-the-day/output/day-053-sfx-tiny-sparks-bounce.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="15" t="n">

</xml_diff>

<commit_message>
Tiny Sparks Marathon #4 (Days 54-57): compile plan, upload kit, thumbnail; tick calendar 54-57
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UgMN9TNxAdhp4UNCAFT25z
</commit_message>
<xml_diff>
--- a/TINY-SPARKS-CALENDAR.xlsx
+++ b/TINY-SPARKS-CALENDAR.xlsx
@@ -6525,7 +6525,7 @@
       </c>
       <c r="Q55" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R55" s="48">
@@ -6541,7 +6541,11 @@
       <c r="V55" s="15" t="n"/>
       <c r="W55" s="15" t="n"/>
       <c r="X55" s="20" t="n"/>
-      <c r="Y55" s="15" t="n"/>
+      <c r="Y55" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-30 → kids-shorts/tiny-sparks/science/day-054-how-does-snow-form/output/day-054-sfx-tiny-sparks-bounce.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="15" t="n">
@@ -6619,7 +6623,7 @@
       </c>
       <c r="Q56" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R56" s="48">
@@ -6635,7 +6639,11 @@
       <c r="V56" s="15" t="n"/>
       <c r="W56" s="15" t="n"/>
       <c r="X56" s="20" t="n"/>
-      <c r="Y56" s="15" t="n"/>
+      <c r="Y56" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-30 → kids-shorts/tiny-sparks/puzzles/day-055-find-the-different-number/output/day-055-sfx-tiny-sparks-bounce.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="15" t="n">
@@ -6713,7 +6721,7 @@
       </c>
       <c r="Q57" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R57" s="48">
@@ -6729,7 +6737,11 @@
       <c r="V57" s="15" t="n"/>
       <c r="W57" s="15" t="n"/>
       <c r="X57" s="20" t="n"/>
-      <c r="Y57" s="15" t="n"/>
+      <c r="Y57" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-30 → kids-shorts/tiny-sparks/songs/day-056-four-seasons-song/output/day-056-final.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="15" t="n">
@@ -6807,7 +6819,7 @@
       </c>
       <c r="Q58" s="15" t="inlineStr">
         <is>
-          <t>Idea</t>
+          <t>Rendered</t>
         </is>
       </c>
       <c r="R58" s="48">
@@ -6823,7 +6835,11 @@
       <c r="V58" s="15" t="n"/>
       <c r="W58" s="15" t="n"/>
       <c r="X58" s="20" t="n"/>
-      <c r="Y58" s="15" t="n"/>
+      <c r="Y58" s="15" t="inlineStr">
+        <is>
+          <t>made 2026-10-30 → kids-shorts/tiny-sparks/stories/day-057-leo-learns-why-we-must-listen/output/day-057-sfx-tiny-sparks-bounce.mp4</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" s="15" t="n">

</xml_diff>